<commit_message>
Final dashboard: format Excel4 and update KPI tables
</commit_message>
<xml_diff>
--- a/excel2.xlsx
+++ b/excel2.xlsx
@@ -1,23 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar-my.sharepoint.com/personal/s_lewis_cgiar_org/Documents/TAAT/R4D/KPIS/zippy/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\IITA2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{787C2D43-E717-4125-AFD9-32FB8B601E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC901A81-6BC2-4922-B6F5-028BF72EA27B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7D6C42FC-A6F5-4FB3-BCAA-02C3B0CCB318}"/>
+    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{31305BA0-5A95-4769-B635-B8A9DFD81AB1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_Hlk200085589" localSheetId="0">Sheet1!#REF!</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -30,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -39,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>KPI Nr</t>
   </si>
@@ -189,15 +184,6 @@
   </si>
   <si>
     <t>Percentage of approved proposals with inclusion of nutrition and health activities</t>
-  </si>
-  <si>
-    <t>Meeting or Exceeding  Target</t>
-  </si>
-  <si>
-    <t>Meeting at least 75% of Target</t>
-  </si>
-  <si>
-    <t>Meeting at least 50% of Target</t>
   </si>
 </sst>
 </file>
@@ -206,29 +192,22 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -237,13 +216,7 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -259,14 +232,13 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="9"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -291,18 +263,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="16">
     <border>
@@ -322,6 +282,43 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -332,7 +329,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -344,24 +341,15 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -371,9 +359,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -384,7 +370,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -397,38 +383,12 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -521,212 +481,196 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="3" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -758,39 +702,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -842,7 +786,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -953,6 +897,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -961,13 +912,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1032,423 +976,385 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{436DF3B9-9B26-4648-BD64-23BB8D8864D3}">
-  <dimension ref="A1:H21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A062B4A-2385-4FE0-A062-3E2553F94E5B}">
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="10.90625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="6.54296875" style="39" customWidth="1"/>
-    <col min="3" max="3" width="35.1796875" style="49" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.1796875" style="66" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.54296875" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.54296875" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" ht="36.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="31" t="s">
+    <row r="1" spans="1:6" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="1"/>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="40" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="57" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="51" t="s">
+    <row r="2" spans="1:6" ht="72" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="14">
+      <c r="D2" s="10">
         <v>272</v>
       </c>
-      <c r="E2" s="58">
+      <c r="E2" s="11">
         <v>220</v>
       </c>
-      <c r="F2" s="15"/>
-      <c r="H2" s="8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="52"/>
-      <c r="B3" s="33" t="s">
+      <c r="F2" s="12"/>
+    </row>
+    <row r="3" spans="1:6" ht="84" x14ac:dyDescent="0.35">
+      <c r="A3" s="13"/>
+      <c r="B3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="42" t="s">
+      <c r="C3" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="16">
         <v>2</v>
       </c>
-      <c r="E3" s="59">
+      <c r="E3" s="17">
         <v>1.3</v>
       </c>
-      <c r="F3" s="16"/>
-      <c r="H3" s="9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" s="3" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="53"/>
-      <c r="B4" s="34" t="s">
+      <c r="F3" s="18"/>
+    </row>
+    <row r="4" spans="1:6" ht="108.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="19"/>
+      <c r="B4" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="43" t="s">
+      <c r="C4" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="17">
+      <c r="D4" s="22">
         <v>1</v>
       </c>
-      <c r="E4" s="60">
+      <c r="E4" s="23">
         <v>6</v>
       </c>
-      <c r="F4" s="18"/>
-      <c r="H4" s="10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="54" t="s">
+      <c r="F4" s="24"/>
+    </row>
+    <row r="5" spans="1:6" ht="72" x14ac:dyDescent="0.35">
+      <c r="A5" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="27">
         <v>150</v>
       </c>
-      <c r="E5" s="61">
+      <c r="E5" s="28">
         <v>113</v>
       </c>
-      <c r="F5" s="22">
+      <c r="F5" s="29">
         <f>67/113</f>
         <v>0.59292035398230092</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="55"/>
-      <c r="B6" s="36" t="s">
+    <row r="6" spans="1:6" ht="72" x14ac:dyDescent="0.35">
+      <c r="A6" s="59"/>
+      <c r="B6" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="45" t="s">
+      <c r="C6" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="32">
         <v>60</v>
       </c>
-      <c r="E6" s="62">
+      <c r="E6" s="33">
         <v>103</v>
       </c>
-      <c r="F6" s="23">
+      <c r="F6" s="34">
         <f>50/103</f>
         <v>0.4854368932038835</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="55"/>
-      <c r="B7" s="36" t="s">
+    <row r="7" spans="1:6" ht="96" x14ac:dyDescent="0.35">
+      <c r="A7" s="59"/>
+      <c r="B7" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="46" t="s">
+      <c r="C7" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="36">
         <v>12000</v>
       </c>
-      <c r="E7" s="62">
+      <c r="E7" s="33">
         <v>12612</v>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="34">
         <v>0.43909999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="3" customFormat="1" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="56"/>
+    <row r="8" spans="1:6" ht="120.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="60"/>
       <c r="B8" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="47" t="s">
+      <c r="C8" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="39">
         <v>150</v>
       </c>
-      <c r="E8" s="63">
+      <c r="E8" s="40">
         <v>1444</v>
       </c>
-      <c r="F8" s="25">
+      <c r="F8" s="41">
         <v>0.33650000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="51" t="s">
+    <row r="9" spans="1:6" ht="24.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="44">
         <v>1</v>
       </c>
-      <c r="E9" s="64">
+      <c r="E9" s="45">
         <v>15</v>
       </c>
-      <c r="F9" s="15"/>
-    </row>
-    <row r="10" spans="1:8" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
-      <c r="B10" s="33" t="s">
+      <c r="F9" s="12"/>
+    </row>
+    <row r="10" spans="1:6" ht="48" x14ac:dyDescent="0.35">
+      <c r="A10" s="62"/>
+      <c r="B10" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="46">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="E10" s="50">
+      <c r="E10" s="47">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="F10" s="16"/>
-    </row>
-    <row r="11" spans="1:8" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
-      <c r="B11" s="33" t="s">
+      <c r="F10" s="18"/>
+    </row>
+    <row r="11" spans="1:6" ht="60" x14ac:dyDescent="0.35">
+      <c r="A11" s="62"/>
+      <c r="B11" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="46" t="s">
+      <c r="C11" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="48">
         <v>1</v>
       </c>
-      <c r="E11" s="65">
+      <c r="E11" s="49">
         <v>1</v>
       </c>
-      <c r="F11" s="16"/>
-    </row>
-    <row r="12" spans="1:8" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="52"/>
-      <c r="B12" s="33" t="s">
+      <c r="F11" s="18"/>
+    </row>
+    <row r="12" spans="1:6" ht="84" x14ac:dyDescent="0.35">
+      <c r="A12" s="62"/>
+      <c r="B12" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="42" t="s">
+      <c r="C12" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="16">
         <v>20</v>
       </c>
-      <c r="E12" s="65">
+      <c r="E12" s="49">
         <v>51</v>
       </c>
-      <c r="F12" s="16"/>
-    </row>
-    <row r="13" spans="1:8" s="3" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="53"/>
-      <c r="B13" s="34" t="s">
+      <c r="F12" s="18"/>
+    </row>
+    <row r="13" spans="1:6" ht="108.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="63"/>
+      <c r="B13" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="43" t="s">
+      <c r="C13" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="17">
+      <c r="D13" s="22">
         <v>30</v>
       </c>
-      <c r="E13" s="60">
+      <c r="E13" s="23">
         <v>19</v>
       </c>
-      <c r="F13" s="18"/>
-    </row>
-    <row r="14" spans="1:8" s="3" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="51" t="s">
+      <c r="F13" s="24"/>
+    </row>
+    <row r="14" spans="1:6" ht="72" x14ac:dyDescent="0.35">
+      <c r="A14" s="61" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="41" t="s">
+      <c r="C14" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="10">
         <v>30</v>
       </c>
-      <c r="E14" s="64">
+      <c r="E14" s="45">
         <v>38</v>
       </c>
-      <c r="F14" s="27"/>
-    </row>
-    <row r="15" spans="1:8" s="3" customFormat="1" ht="12" x14ac:dyDescent="0.25">
-      <c r="A15" s="52"/>
-      <c r="B15" s="33" t="s">
+      <c r="F14" s="50"/>
+    </row>
+    <row r="15" spans="1:6" ht="48" x14ac:dyDescent="0.35">
+      <c r="A15" s="62"/>
+      <c r="B15" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="42" t="s">
+      <c r="C15" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="16">
         <v>30</v>
       </c>
-      <c r="E15" s="65">
+      <c r="E15" s="49">
         <v>83</v>
       </c>
-      <c r="F15" s="28"/>
-    </row>
-    <row r="16" spans="1:8" s="3" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A16" s="52"/>
-      <c r="B16" s="33" t="s">
+      <c r="F15" s="51"/>
+    </row>
+    <row r="16" spans="1:6" ht="72" x14ac:dyDescent="0.35">
+      <c r="A16" s="62"/>
+      <c r="B16" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="42" t="s">
+      <c r="C16" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="16">
         <v>30</v>
       </c>
-      <c r="E16" s="65">
+      <c r="E16" s="49">
         <v>8</v>
       </c>
-      <c r="F16" s="16"/>
-    </row>
-    <row r="17" spans="1:6" s="3" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A17" s="52"/>
-      <c r="B17" s="33" t="s">
+      <c r="F16" s="18"/>
+    </row>
+    <row r="17" spans="1:6" ht="96" x14ac:dyDescent="0.35">
+      <c r="A17" s="62"/>
+      <c r="B17" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="42" t="s">
+      <c r="C17" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="16">
         <v>30</v>
       </c>
-      <c r="E17" s="65">
+      <c r="E17" s="49">
         <v>18</v>
       </c>
-      <c r="F17" s="16"/>
-    </row>
-    <row r="18" spans="1:6" s="3" customFormat="1" ht="36.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="53"/>
-      <c r="B18" s="34" t="s">
+      <c r="F17" s="18"/>
+    </row>
+    <row r="18" spans="1:6" ht="180.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="63"/>
+      <c r="B18" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="47" t="s">
+      <c r="C18" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="D18" s="17">
+      <c r="D18" s="22">
         <v>30</v>
       </c>
-      <c r="E18" s="60">
+      <c r="E18" s="23">
         <v>12</v>
       </c>
-      <c r="F18" s="18"/>
-    </row>
-    <row r="19" spans="1:6" s="3" customFormat="1" ht="30.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="51" t="s">
+      <c r="F18" s="24"/>
+    </row>
+    <row r="19" spans="1:6" ht="120" x14ac:dyDescent="0.35">
+      <c r="A19" s="61" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="32" t="s">
+      <c r="B19" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="41" t="s">
+      <c r="C19" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D19" s="29">
+      <c r="D19" s="52">
         <v>0.25</v>
       </c>
-      <c r="E19" s="67">
+      <c r="E19" s="53">
         <v>0.41666666666666669</v>
       </c>
-      <c r="F19" s="15"/>
-    </row>
-    <row r="20" spans="1:6" s="3" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A20" s="52"/>
-      <c r="B20" s="33" t="s">
+      <c r="F19" s="12"/>
+    </row>
+    <row r="20" spans="1:6" ht="108" x14ac:dyDescent="0.35">
+      <c r="A20" s="62"/>
+      <c r="B20" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="C20" s="42" t="s">
+      <c r="C20" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="54">
         <v>0.25</v>
       </c>
-      <c r="E20" s="68">
+      <c r="E20" s="55">
         <v>0.3611111111111111</v>
       </c>
-      <c r="F20" s="16"/>
-    </row>
-    <row r="21" spans="1:6" s="3" customFormat="1" ht="24.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="53"/>
-      <c r="B21" s="34" t="s">
+      <c r="F20" s="18"/>
+    </row>
+    <row r="21" spans="1:6" ht="108.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="63"/>
+      <c r="B21" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="43" t="s">
+      <c r="C21" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="D21" s="30">
+      <c r="D21" s="56">
         <v>0.25</v>
       </c>
-      <c r="E21" s="69">
+      <c r="E21" s="57">
         <v>0.1111111111111111</v>
       </c>
-      <c r="F21" s="18"/>
+      <c r="F21" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A19:A21"/>
-    <mergeCell ref="A2:A4"/>
+  <mergeCells count="4">
     <mergeCell ref="A5:A8"/>
     <mergeCell ref="A9:A13"/>
     <mergeCell ref="A14:A18"/>
+    <mergeCell ref="A19:A21"/>
   </mergeCells>
   <conditionalFormatting sqref="E2">
     <cfRule type="colorScale" priority="20">
@@ -1687,6 +1593,5 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>